<commit_message>
Add dataset supporting Turbo Expo and JEGTP publications
</commit_message>
<xml_diff>
--- a/Validation/ValidationData.xlsx
+++ b/Validation/ValidationData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b266c95a83fbf4bb/Documenten/TU Delft Aerospace Engineering/Msc2/AE5222 - Thesis/Software/Conceptual-Investigation-of-Alternative-Electric-Ducted-Fan-Architectures/Validation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tud365-my.sharepoint.com/personal/thomasvermeule_tudelft_nl/Documents/Documents/UDC and Optimisation Framework/AircraftDuctedFanOptimisation/Validation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1630" documentId="8_{E7BF6703-466F-4498-AEEA-FFB8403C4F5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9A69BF3-03B0-4F84-A66A-288E19B964EF}"/>
+  <xr:revisionPtr revIDLastSave="1638" documentId="8_{E7BF6703-466F-4498-AEEA-FFB8403C4F5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82AA3A58-F464-5B7D-9A8D-57D84482FC8B}"/>
   <bookViews>
-    <workbookView xWindow="43800" yWindow="2590" windowWidth="28800" windowHeight="15200" firstSheet="2" activeTab="3" xr2:uid="{6111FCF9-37F3-4199-9E4E-EEB7F0803D9A}"/>
+    <workbookView xWindow="6480" yWindow="11160" windowWidth="21600" windowHeight="11295" firstSheet="2" activeTab="3" xr2:uid="{6111FCF9-37F3-4199-9E4E-EEB7F0803D9A}"/>
   </bookViews>
   <sheets>
     <sheet name="Wind Tunnel Beta=29deg data" sheetId="16" r:id="rId1"/>
@@ -16980,24 +16980,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B26E69B-6441-4D2A-91E2-CF3588D774EF}">
   <dimension ref="A1:L12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -17005,7 +17005,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -17037,7 +17037,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>0.3</v>
       </c>
@@ -17076,7 +17076,7 @@
         <v>0.74074074074074081</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>0.35</v>
       </c>
@@ -17115,7 +17115,7 @@
         <v>0.46647230320699723</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>0.4</v>
       </c>
@@ -17154,7 +17154,7 @@
         <v>0.31249999999999994</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>0.45</v>
       </c>
@@ -17193,7 +17193,7 @@
         <v>0.21947873799725648</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>0.5</v>
       </c>
@@ -17232,7 +17232,7 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>0.55000000000000004</v>
       </c>
@@ -17271,7 +17271,7 @@
         <v>0.12021036814425241</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>0.6</v>
       </c>
@@ -17327,24 +17327,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CBD950F-5FB4-419F-B6AE-C3E6C12B06BE}">
   <dimension ref="A1:L12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -17352,7 +17352,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -17384,7 +17384,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>0.3</v>
       </c>
@@ -17423,7 +17423,7 @@
         <v>0.74074074074074081</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>0.35</v>
       </c>
@@ -17462,7 +17462,7 @@
         <v>0.46647230320699723</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>0.4</v>
       </c>
@@ -17501,7 +17501,7 @@
         <v>0.31249999999999994</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>0.45</v>
       </c>
@@ -17540,7 +17540,7 @@
         <v>0.21947873799725648</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>0.5</v>
       </c>
@@ -17579,7 +17579,7 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>0.55000000000000004</v>
       </c>
@@ -17618,7 +17618,7 @@
         <v>0.12021036814425241</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>0.6</v>
       </c>
@@ -17674,12 +17674,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D17483C-FDF0-45AC-9867-0493571C96AF}">
   <dimension ref="F1:AO19"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="15" max="15" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="6:41" x14ac:dyDescent="0.35">
+    <row r="1" spans="6:41" x14ac:dyDescent="0.25">
       <c r="F1" t="s">
         <v>2</v>
       </c>
@@ -17700,7 +17700,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="6:41" x14ac:dyDescent="0.35">
+    <row r="2" spans="6:41" x14ac:dyDescent="0.25">
       <c r="F2" t="s">
         <v>3</v>
       </c>
@@ -17727,7 +17727,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="6:41" x14ac:dyDescent="0.35">
+    <row r="3" spans="6:41" x14ac:dyDescent="0.25">
       <c r="F3">
         <f>H3*2*PI()*$P$1/G3</f>
         <v>20.943951023931955</v>
@@ -17751,7 +17751,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="6:41" x14ac:dyDescent="0.35">
+    <row r="4" spans="6:41" x14ac:dyDescent="0.25">
       <c r="F4">
         <f t="shared" ref="F4:F9" si="0">H4*2*PI()*$P$1/G4</f>
         <v>17.951958020513104</v>
@@ -17775,7 +17775,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="6:41" x14ac:dyDescent="0.35">
+    <row r="5" spans="6:41" x14ac:dyDescent="0.25">
       <c r="F5">
         <f t="shared" si="0"/>
         <v>15.707963267948966</v>
@@ -17801,7 +17801,7 @@
         <v>0.66311381150987769</v>
       </c>
     </row>
-    <row r="6" spans="6:41" x14ac:dyDescent="0.35">
+    <row r="6" spans="6:41" x14ac:dyDescent="0.25">
       <c r="F6">
         <f t="shared" si="0"/>
         <v>13.962634015954636</v>
@@ -17825,7 +17825,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="7" spans="6:41" x14ac:dyDescent="0.35">
+    <row r="7" spans="6:41" x14ac:dyDescent="0.25">
       <c r="F7">
         <f t="shared" si="0"/>
         <v>12.566370614359172</v>
@@ -17851,7 +17851,7 @@
         <v>0.7222979181849869</v>
       </c>
     </row>
-    <row r="8" spans="6:41" x14ac:dyDescent="0.35">
+    <row r="8" spans="6:41" x14ac:dyDescent="0.25">
       <c r="F8">
         <f t="shared" si="0"/>
         <v>11.423973285781065</v>
@@ -17877,7 +17877,7 @@
         <v>0.73735942999399084</v>
       </c>
     </row>
-    <row r="9" spans="6:41" x14ac:dyDescent="0.35">
+    <row r="9" spans="6:41" x14ac:dyDescent="0.25">
       <c r="F9">
         <f t="shared" si="0"/>
         <v>10.471975511965978</v>
@@ -17906,7 +17906,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="6:41" ht="65.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="6:41" ht="65.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="AG10" s="8" t="s">
         <v>29</v>
       </c>
@@ -17919,7 +17919,7 @@
       <c r="AN10" s="8"/>
       <c r="AO10" s="8"/>
     </row>
-    <row r="11" spans="6:41" x14ac:dyDescent="0.35">
+    <row r="11" spans="6:41" x14ac:dyDescent="0.25">
       <c r="F11" t="s">
         <v>2</v>
       </c>
@@ -17936,7 +17936,7 @@
       <c r="AN11" s="8"/>
       <c r="AO11" s="8"/>
     </row>
-    <row r="12" spans="6:41" x14ac:dyDescent="0.35">
+    <row r="12" spans="6:41" x14ac:dyDescent="0.25">
       <c r="F12" t="s">
         <v>3</v>
       </c>
@@ -17959,7 +17959,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="6:41" x14ac:dyDescent="0.35">
+    <row r="13" spans="6:41" x14ac:dyDescent="0.25">
       <c r="F13">
         <f>H13*2*PI()*$P$1/G13</f>
         <v>20.943951023931955</v>
@@ -17979,7 +17979,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="14" spans="6:41" x14ac:dyDescent="0.35">
+    <row r="14" spans="6:41" x14ac:dyDescent="0.25">
       <c r="F14">
         <f t="shared" ref="F14:F19" si="3">H14*2*PI()*$P$1/G14</f>
         <v>17.951958020513104</v>
@@ -18005,7 +18005,7 @@
         <v>0.68237501065855666</v>
       </c>
     </row>
-    <row r="15" spans="6:41" x14ac:dyDescent="0.35">
+    <row r="15" spans="6:41" x14ac:dyDescent="0.25">
       <c r="F15">
         <f t="shared" si="3"/>
         <v>15.707963267948966</v>
@@ -18031,7 +18031,7 @@
         <v>0.73950214916631241</v>
       </c>
     </row>
-    <row r="16" spans="6:41" x14ac:dyDescent="0.35">
+    <row r="16" spans="6:41" x14ac:dyDescent="0.25">
       <c r="F16">
         <f t="shared" si="3"/>
         <v>13.962634015954636</v>
@@ -18057,7 +18057,7 @@
         <v>0.783448275862069</v>
       </c>
     </row>
-    <row r="17" spans="6:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="6:12" x14ac:dyDescent="0.25">
       <c r="F17">
         <f t="shared" si="3"/>
         <v>12.566370614359172</v>
@@ -18083,7 +18083,7 @@
         <v>0.8144490579683038</v>
       </c>
     </row>
-    <row r="18" spans="6:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="6:12" x14ac:dyDescent="0.25">
       <c r="F18">
         <f t="shared" si="3"/>
         <v>11.423973285781065</v>
@@ -18109,7 +18109,7 @@
         <v>0.82430531487635328</v>
       </c>
     </row>
-    <row r="19" spans="6:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="6:12" x14ac:dyDescent="0.25">
       <c r="F19">
         <f t="shared" si="3"/>
         <v>10.471975511965978</v>
@@ -18150,12 +18150,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC9A3C9B-DBC3-40D2-A144-241D094FABD6}">
   <dimension ref="F1:AA19"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="16" max="16" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="6:27" x14ac:dyDescent="0.35">
+    <row r="1" spans="6:27" x14ac:dyDescent="0.25">
       <c r="F1" t="s">
         <v>2</v>
       </c>
@@ -18176,7 +18176,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="6:27" x14ac:dyDescent="0.35">
+    <row r="2" spans="6:27" x14ac:dyDescent="0.25">
       <c r="F2" t="s">
         <v>3</v>
       </c>
@@ -18215,7 +18215,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="6:27" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="6:27" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F3">
         <f t="shared" ref="F3:F5" si="0">H3*2*PI()*$Q$1/G3</f>
         <v>20.943951023931955</v>
@@ -18257,7 +18257,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="6:27" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="6:27" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F4">
         <f t="shared" si="0"/>
         <v>17.951958020513104</v>
@@ -18301,7 +18301,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="6:27" x14ac:dyDescent="0.35">
+    <row r="5" spans="6:27" x14ac:dyDescent="0.25">
       <c r="F5">
         <f t="shared" si="0"/>
         <v>15.707963267948967</v>
@@ -18347,7 +18347,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="6:27" x14ac:dyDescent="0.35">
+    <row r="6" spans="6:27" x14ac:dyDescent="0.25">
       <c r="F6">
         <f>H6*2*PI()*$Q$1/G6</f>
         <v>13.962634015954636</v>
@@ -18389,7 +18389,7 @@
         <v>1.4158256249999973E-2</v>
       </c>
     </row>
-    <row r="7" spans="6:27" x14ac:dyDescent="0.35">
+    <row r="7" spans="6:27" x14ac:dyDescent="0.25">
       <c r="F7">
         <f t="shared" ref="F7:F8" si="4">H7*2*PI()*$Q$1/G7</f>
         <v>12.566370614359174</v>
@@ -18431,7 +18431,7 @@
         <v>1.683125000000002E-2</v>
       </c>
     </row>
-    <row r="8" spans="6:27" x14ac:dyDescent="0.35">
+    <row r="8" spans="6:27" x14ac:dyDescent="0.25">
       <c r="F8">
         <f t="shared" si="4"/>
         <v>11.423973285781063</v>
@@ -18473,7 +18473,7 @@
         <v>1.4864899999999931E-2</v>
       </c>
     </row>
-    <row r="9" spans="6:27" x14ac:dyDescent="0.35">
+    <row r="9" spans="6:27" x14ac:dyDescent="0.25">
       <c r="F9">
         <f>H9*2*PI()*$Q$1/G9</f>
         <v>10.471975511965978</v>
@@ -18515,7 +18515,7 @@
         <v>1.189160000000003E-2</v>
       </c>
     </row>
-    <row r="11" spans="6:27" x14ac:dyDescent="0.35">
+    <row r="11" spans="6:27" x14ac:dyDescent="0.25">
       <c r="F11" t="s">
         <v>2</v>
       </c>
@@ -18523,7 +18523,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="6:27" x14ac:dyDescent="0.35">
+    <row r="12" spans="6:27" x14ac:dyDescent="0.25">
       <c r="F12" t="s">
         <v>3</v>
       </c>
@@ -18558,7 +18558,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="6:27" x14ac:dyDescent="0.35">
+    <row r="13" spans="6:27" x14ac:dyDescent="0.25">
       <c r="F13">
         <f t="shared" ref="F13" si="6">H13*2*PI()*$Q$1/G13</f>
         <v>20.943951023931955</v>
@@ -18600,7 +18600,7 @@
         <v>9.9375000000000158E-3</v>
       </c>
     </row>
-    <row r="14" spans="6:27" x14ac:dyDescent="0.35">
+    <row r="14" spans="6:27" x14ac:dyDescent="0.25">
       <c r="F14">
         <f t="shared" ref="F14:F19" si="8">H14*2*PI()*$Q$1/G14</f>
         <v>17.951958020513104</v>
@@ -18642,7 +18642,7 @@
         <v>1.1584400000000022E-2</v>
       </c>
     </row>
-    <row r="15" spans="6:27" x14ac:dyDescent="0.35">
+    <row r="15" spans="6:27" x14ac:dyDescent="0.25">
       <c r="F15">
         <f t="shared" si="8"/>
         <v>15.707963267948967</v>
@@ -18684,7 +18684,7 @@
         <v>1.3574399999999986E-2</v>
       </c>
     </row>
-    <row r="16" spans="6:27" x14ac:dyDescent="0.35">
+    <row r="16" spans="6:27" x14ac:dyDescent="0.25">
       <c r="F16">
         <f t="shared" si="8"/>
         <v>13.962634015954636</v>
@@ -18726,7 +18726,7 @@
         <v>1.6719256249999988E-2</v>
       </c>
     </row>
-    <row r="17" spans="6:16" x14ac:dyDescent="0.35">
+    <row r="17" spans="6:16" x14ac:dyDescent="0.25">
       <c r="F17">
         <f t="shared" si="8"/>
         <v>12.566370614359174</v>
@@ -18768,7 +18768,7 @@
         <v>1.7923749999999995E-2</v>
       </c>
     </row>
-    <row r="18" spans="6:16" x14ac:dyDescent="0.35">
+    <row r="18" spans="6:16" x14ac:dyDescent="0.25">
       <c r="F18">
         <f t="shared" si="8"/>
         <v>11.423973285781063</v>
@@ -18810,7 +18810,7 @@
         <v>1.9139467499999986E-2</v>
       </c>
     </row>
-    <row r="19" spans="6:16" x14ac:dyDescent="0.35">
+    <row r="19" spans="6:16" x14ac:dyDescent="0.25">
       <c r="F19">
         <f t="shared" si="8"/>
         <v>10.471975511965978</v>

</xml_diff>